<commit_message>
codigo y documentacion actualizada a 202603
</commit_message>
<xml_diff>
--- a/Energia/A2_Structure_Lists.xlsx
+++ b/Energia/A2_Structure_Lists.xlsx
@@ -1213,25 +1213,25 @@
     <t>DEMTRN_NOMOT</t>
   </si>
   <si>
+    <t>CO2_scc</t>
+  </si>
+  <si>
+    <t>Accidents</t>
+  </si>
+  <si>
+    <t>CO2_fugitivas_scc</t>
+  </si>
+  <si>
+    <t>Congestion</t>
+  </si>
+  <si>
     <t>Health</t>
   </si>
   <si>
+    <t>CO2</t>
+  </si>
+  <si>
     <t>CO2_fugitivas</t>
-  </si>
-  <si>
-    <t>CO2</t>
-  </si>
-  <si>
-    <t>Congestion</t>
-  </si>
-  <si>
-    <t>CO2_scc</t>
-  </si>
-  <si>
-    <t>Accidents</t>
-  </si>
-  <si>
-    <t>CO2_fugitivas_scc</t>
   </si>
   <si>
     <t>ECU</t>

</xml_diff>